<commit_message>
cineagent experiments syntax updated
</commit_message>
<xml_diff>
--- a/evaluation_tests/cineagent_evaluation.xlsx
+++ b/evaluation_tests/cineagent_evaluation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sasoffice365-my.sharepoint.com/personal/stefano_podofillini_sas_com/Documents/Documents/Projects/internal/sas-ram-hackathon/evaluation_tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_69D1F52FB4F8C43E299834C2FD56468A962AC24F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_69D1F52FB4F8C43E299834C2FD56468A962AC24F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ECA2B16C-0B31-47C5-B0B0-B53AC1545E1B}"/>
   <bookViews>
     <workbookView xWindow="4650" yWindow="1740" windowWidth="27090" windowHeight="17220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,10 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="73">
-  <si>
-    <t>RAG Evaluation Test 3 - Agent with Data and Documents</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="71">
   <si>
     <t>10 questions covering document retrieval, structured-data retrieval, guideline compliance, cross-source reasoning, and temporal reasoning.</t>
   </si>
@@ -130,12 +127,6 @@
     <t>Budget: 19000000; revenue: 46998772.</t>
   </si>
   <si>
-    <t>19000000</t>
-  </si>
-  <si>
-    <t>46998772</t>
-  </si>
-  <si>
     <t>movies_abt_v2 1.xlsx</t>
   </si>
   <si>
@@ -145,9 +136,6 @@
     <t>06/13/1980.</t>
   </si>
   <si>
-    <t>06/13/1980</t>
-  </si>
-  <si>
     <t>What genre and rating are recorded for The Shining?</t>
   </si>
   <si>
@@ -239,12 +227,21 @@
   </si>
   <si>
     <t>awards</t>
+  </si>
+  <si>
+    <t>13 June 1980</t>
+  </si>
+  <si>
+    <t>Evaluation Tests - CineAgent</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
+  </numFmts>
   <fonts count="4">
     <font>
       <sz val="11"/>
@@ -304,7 +301,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -316,6 +313,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -520,7 +523,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="30" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -537,7 +540,7 @@
     </row>
     <row r="2" spans="1:13" ht="30" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
@@ -554,43 +557,43 @@
     </row>
     <row r="4" spans="1:13" ht="15">
       <c r="A4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="I4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="J4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="K4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="L4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="L4" s="1" t="s">
+      <c r="M4" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="48" customHeight="1">
@@ -598,34 +601,34 @@
         <v>1</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>20</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>21</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M5" s="2" t="s">
         <v>22</v>
-      </c>
-      <c r="M5" s="2" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="48" customHeight="1">
@@ -633,36 +636,36 @@
         <v>2</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F6" s="2" t="s">
+      <c r="G6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H6" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="H6" s="2" t="s">
+      <c r="I6" s="2" t="s">
         <v>27</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>28</v>
       </c>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
       <c r="L6" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="48" customHeight="1">
@@ -670,19 +673,19 @@
         <v>3</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C7" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="E7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>32</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
@@ -690,10 +693,10 @@
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
       <c r="L7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M7" s="2" t="s">
         <v>22</v>
-      </c>
-      <c r="M7" s="2" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="48" customHeight="1">
@@ -701,34 +704,34 @@
         <v>4</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>35</v>
-      </c>
       <c r="E8" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>36</v>
+        <v>17</v>
+      </c>
+      <c r="F8" s="5">
+        <v>19000000</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>37</v>
+        <v>19</v>
+      </c>
+      <c r="H8" s="5">
+        <v>46998772</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
       <c r="L8" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="48" customHeight="1">
@@ -736,19 +739,19 @@
         <v>5</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>41</v>
+        <v>17</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>69</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
@@ -756,10 +759,10 @@
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
       <c r="L9" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="48" customHeight="1">
@@ -767,34 +770,34 @@
         <v>6</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
       <c r="L10" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="48" customHeight="1">
@@ -802,34 +805,34 @@
         <v>7</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="G11" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H11" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>51</v>
       </c>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
       <c r="L11" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="48" customHeight="1">
@@ -837,34 +840,34 @@
         <v>8</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H12" s="2" t="s">
         <v>53</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>57</v>
       </c>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="48" customHeight="1">
@@ -872,38 +875,38 @@
         <v>9</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C13" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="I13" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="J13" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>64</v>
       </c>
       <c r="K13" s="2"/>
       <c r="L13" s="2" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="48" customHeight="1">
@@ -911,40 +914,40 @@
         <v>10</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H14" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="I14" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="J14" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="K14" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="E14" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="K14" s="2" t="s">
-        <v>72</v>
-      </c>
       <c r="L14" s="2" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated test syntax and system prompts
</commit_message>
<xml_diff>
--- a/evaluation_tests/cineagent_evaluation.xlsx
+++ b/evaluation_tests/cineagent_evaluation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sasoffice365-my.sharepoint.com/personal/stefano_podofillini_sas_com/Documents/Documents/Projects/internal/sas-ram-hackathon/evaluation_tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_69D1F52FB4F8C43E299834C2FD56468A962AC24F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ECA2B16C-0B31-47C5-B0B0-B53AC1545E1B}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="11_69D1F52FB4F8C43E299834C2FD56468A962AC24F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{80042DA0-508D-4AAC-8B7F-419166DBA76E}"/>
   <bookViews>
     <workbookView xWindow="4650" yWindow="1740" windowWidth="27090" windowHeight="17220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -121,9 +121,6 @@
     <t>Structured data retrieval</t>
   </si>
   <si>
-    <t>What are the budget and revenue of The Shining?</t>
-  </si>
-  <si>
     <t>Budget: 19000000; revenue: 46998772.</t>
   </si>
   <si>
@@ -233,6 +230,9 @@
   </si>
   <si>
     <t>Evaluation Tests - CineAgent</t>
+  </si>
+  <si>
+    <t>Using only information you can retrieve from RAG and MCP, answer the following question: what are the budget and revenue of The Shining?</t>
   </si>
 </sst>
 </file>
@@ -309,16 +309,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -336,6 +336,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -522,38 +526,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="30" customHeight="1">
-      <c r="A1" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
+      <c r="A1" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="5"/>
+      <c r="K1" s="5"/>
+      <c r="L1" s="5"/>
+      <c r="M1" s="5"/>
     </row>
     <row r="2" spans="1:13" ht="30" customHeight="1">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="6"/>
+      <c r="K2" s="6"/>
+      <c r="L2" s="6"/>
+      <c r="M2" s="6"/>
     </row>
     <row r="4" spans="1:13" ht="15">
       <c r="A4" s="1" t="s">
@@ -707,21 +711,21 @@
         <v>32</v>
       </c>
       <c r="C8" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>33</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>34</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="3">
         <v>19000000</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="H8" s="5">
+      <c r="H8" s="3">
         <v>46998772</v>
       </c>
       <c r="I8" s="2"/>
@@ -731,7 +735,7 @@
         <v>28</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="48" customHeight="1">
@@ -742,16 +746,16 @@
         <v>32</v>
       </c>
       <c r="C9" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>37</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="6" t="s">
-        <v>69</v>
+      <c r="F9" s="4" t="s">
+        <v>68</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
@@ -762,7 +766,7 @@
         <v>21</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="48" customHeight="1">
@@ -773,22 +777,22 @@
         <v>32</v>
       </c>
       <c r="C10" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>39</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>19</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
@@ -797,7 +801,7 @@
         <v>28</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="48" customHeight="1">
@@ -805,25 +809,25 @@
         <v>7</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="F11" s="2" t="s">
         <v>45</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>46</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>19</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
@@ -832,7 +836,7 @@
         <v>28</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="48" customHeight="1">
@@ -840,25 +844,25 @@
         <v>8</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="E12" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>51</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>52</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>19</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
@@ -867,7 +871,7 @@
         <v>28</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="48" customHeight="1">
@@ -875,38 +879,38 @@
         <v>9</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C13" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>55</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>56</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>19</v>
       </c>
       <c r="H13" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="I13" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="I13" s="2" t="s">
+      <c r="J13" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>60</v>
       </c>
       <c r="K13" s="2"/>
       <c r="L13" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="48" customHeight="1">
@@ -914,40 +918,40 @@
         <v>10</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="E14" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>65</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>19</v>
       </c>
       <c r="H14" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="J14" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I14" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="J14" s="2" t="s">
+      <c r="K14" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="K14" s="2" t="s">
-        <v>68</v>
-      </c>
       <c r="L14" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>